<commit_message>
Cache computed values in the part summary workbook
LibreOffice cannot start in this environment, so openpyxl's formula cells
had no cached results and read back as blank in previewers and pandas.
Injected the computed value into all 30 formula cells; the formulas are
unchanged and Excel still recalculates on open (fullCalcOnLoad).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013cUXqDDQfDDorAWa33JviH
</commit_message>
<xml_diff>
--- a/output/Part_Summary_Wistron_VV726800136.xlsx
+++ b/output/Part_Summary_Wistron_VV726800136.xlsx
@@ -798,14 +798,17 @@
       </c>
       <c r="I12" s="9">
         <f>G12*H12</f>
+        <v>120122.4</v>
         <v/>
       </c>
       <c r="J12" s="10">
         <f>G12*INDEX('Packing list'!$C$4:$C$8,MATCH(F12,'Packing list'!$A$4:$A$8,0))/INDEX('Packing list'!$B$4:$B$8,MATCH(F12,'Packing list'!$A$4:$A$8,0))</f>
+        <v>142.32</v>
         <v/>
       </c>
       <c r="K12" s="10">
         <f>G12*INDEX('Packing list'!$D$4:$D$8,MATCH(F12,'Packing list'!$A$4:$A$8,0))/INDEX('Packing list'!$B$4:$B$8,MATCH(F12,'Packing list'!$A$4:$A$8,0))</f>
+        <v>225</v>
         <v/>
       </c>
       <c r="L12" s="5" t="inlineStr">
@@ -853,14 +856,17 @@
       </c>
       <c r="I13" s="9">
         <f>G13*H13</f>
+        <v>74722.56</v>
         <v/>
       </c>
       <c r="J13" s="10">
         <f>G13*INDEX('Packing list'!$C$4:$C$8,MATCH(F13,'Packing list'!$A$4:$A$8,0))/INDEX('Packing list'!$B$4:$B$8,MATCH(F13,'Packing list'!$A$4:$A$8,0))</f>
+        <v>96</v>
         <v/>
       </c>
       <c r="K13" s="10">
         <f>G13*INDEX('Packing list'!$D$4:$D$8,MATCH(F13,'Packing list'!$A$4:$A$8,0))/INDEX('Packing list'!$B$4:$B$8,MATCH(F13,'Packing list'!$A$4:$A$8,0))</f>
+        <v>166</v>
         <v/>
       </c>
       <c r="L13" s="5" t="inlineStr">
@@ -908,14 +914,17 @@
       </c>
       <c r="I14" s="9">
         <f>G14*H14</f>
+        <v>5310.76</v>
         <v/>
       </c>
       <c r="J14" s="10">
         <f>G14*INDEX('Packing list'!$C$4:$C$8,MATCH(F14,'Packing list'!$A$4:$A$8,0))/INDEX('Packing list'!$B$4:$B$8,MATCH(F14,'Packing list'!$A$4:$A$8,0))</f>
+        <v>6.6076705882</v>
         <v/>
       </c>
       <c r="K14" s="10">
         <f>G14*INDEX('Packing list'!$D$4:$D$8,MATCH(F14,'Packing list'!$A$4:$A$8,0))/INDEX('Packing list'!$B$4:$B$8,MATCH(F14,'Packing list'!$A$4:$A$8,0))</f>
+        <v>19.4044117647</v>
         <v/>
       </c>
       <c r="L14" s="5" t="inlineStr">
@@ -963,14 +972,17 @@
       </c>
       <c r="I15" s="9">
         <f>G15*H15</f>
+        <v>15807.96</v>
         <v/>
       </c>
       <c r="J15" s="10">
         <f>G15*INDEX('Packing list'!$C$4:$C$8,MATCH(F15,'Packing list'!$A$4:$A$8,0))/INDEX('Packing list'!$B$4:$B$8,MATCH(F15,'Packing list'!$A$4:$A$8,0))</f>
+        <v>13.7236235294</v>
         <v/>
       </c>
       <c r="K15" s="10">
         <f>G15*INDEX('Packing list'!$D$4:$D$8,MATCH(F15,'Packing list'!$A$4:$A$8,0))/INDEX('Packing list'!$B$4:$B$8,MATCH(F15,'Packing list'!$A$4:$A$8,0))</f>
+        <v>40.3014705882</v>
         <v/>
       </c>
       <c r="L15" s="5" t="inlineStr">
@@ -1018,14 +1030,17 @@
       </c>
       <c r="I16" s="9">
         <f>G16*H16</f>
+        <v>42518.4</v>
         <v/>
       </c>
       <c r="J16" s="10">
         <f>G16*INDEX('Packing list'!$C$4:$C$8,MATCH(F16,'Packing list'!$A$4:$A$8,0))/INDEX('Packing list'!$B$4:$B$8,MATCH(F16,'Packing list'!$A$4:$A$8,0))</f>
+        <v>4.3567058824</v>
         <v/>
       </c>
       <c r="K16" s="10">
         <f>G16*INDEX('Packing list'!$D$4:$D$8,MATCH(F16,'Packing list'!$A$4:$A$8,0))/INDEX('Packing list'!$B$4:$B$8,MATCH(F16,'Packing list'!$A$4:$A$8,0))</f>
+        <v>12.7941176471</v>
         <v/>
       </c>
       <c r="L16" s="5" t="inlineStr">
@@ -1073,14 +1088,17 @@
       </c>
       <c r="I17" s="9">
         <f>G17*H17</f>
+        <v>5230.8</v>
         <v/>
       </c>
       <c r="J17" s="10">
         <f>G17*INDEX('Packing list'!$C$4:$C$8,MATCH(F17,'Packing list'!$A$4:$A$8,0))/INDEX('Packing list'!$B$4:$B$8,MATCH(F17,'Packing list'!$A$4:$A$8,0))</f>
+        <v>9</v>
         <v/>
       </c>
       <c r="K17" s="10">
         <f>G17*INDEX('Packing list'!$D$4:$D$8,MATCH(F17,'Packing list'!$A$4:$A$8,0))/INDEX('Packing list'!$B$4:$B$8,MATCH(F17,'Packing list'!$A$4:$A$8,0))</f>
+        <v>33</v>
         <v/>
       </c>
       <c r="L17" s="5" t="inlineStr">
@@ -1128,14 +1146,17 @@
       </c>
       <c r="I18" s="9">
         <f>G18*H18</f>
+        <v>24665.76</v>
         <v/>
       </c>
       <c r="J18" s="10">
         <f>G18*INDEX('Packing list'!$C$4:$C$8,MATCH(F18,'Packing list'!$A$4:$A$8,0))/INDEX('Packing list'!$B$4:$B$8,MATCH(F18,'Packing list'!$A$4:$A$8,0))</f>
+        <v>50.4</v>
         <v/>
       </c>
       <c r="K18" s="10">
         <f>G18*INDEX('Packing list'!$D$4:$D$8,MATCH(F18,'Packing list'!$A$4:$A$8,0))/INDEX('Packing list'!$B$4:$B$8,MATCH(F18,'Packing list'!$A$4:$A$8,0))</f>
+        <v>100</v>
         <v/>
       </c>
       <c r="L18" s="5" t="inlineStr">
@@ -1161,19 +1182,23 @@
       <c r="F19" s="12" t="n"/>
       <c r="G19" s="13">
         <f>SUM(G12:G18)</f>
+        <v>2500</v>
         <v/>
       </c>
       <c r="H19" s="12" t="n"/>
       <c r="I19" s="14">
         <f>SUM(I12:I18)</f>
+        <v>288378.64</v>
         <v/>
       </c>
       <c r="J19" s="15">
         <f>SUM(J12:J18)</f>
+        <v>322.408</v>
         <v/>
       </c>
       <c r="K19" s="15">
         <f>SUM(K12:K18)</f>
+        <v>596.5</v>
         <v/>
       </c>
       <c r="L19" s="12" t="n"/>
@@ -1186,6 +1211,7 @@
       </c>
       <c r="G21" s="17">
         <f>I19</f>
+        <v>288378.64</v>
         <v/>
       </c>
     </row>
@@ -1448,18 +1474,22 @@
       </c>
       <c r="B9" s="13">
         <f>SUM(B4:B8)</f>
+        <v>2500</v>
         <v/>
       </c>
       <c r="C9" s="15">
         <f>SUM(C4:C8)</f>
+        <v>322.408</v>
         <v/>
       </c>
       <c r="D9" s="15">
         <f>SUM(D4:D8)</f>
+        <v>596.5</v>
         <v/>
       </c>
       <c r="E9" s="12">
         <f>SUM(E4:E8)</f>
+        <v>76</v>
         <v/>
       </c>
       <c r="F9" s="12" t="n"/>

</xml_diff>